<commit_message>
Update shared export template and submitter example
</commit_message>
<xml_diff>
--- a/CC_Codex 用户满意度标注（试标）.xlsx
+++ b/CC_Codex 用户满意度标注（试标）.xlsx
@@ -15,7 +15,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy/MM/dd HH:mm"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -26,6 +29,13 @@
       <sz val="10"/>
       <color/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="DengXian"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -49,10 +59,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="false">
+      <alignment/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="false">
+      <alignment/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -348,6 +364,8 @@
     <col min="23" max="23" width="19" customWidth="1"/>
     <col min="24" max="24" width="19" customWidth="1"/>
     <col min="25" max="25" width="19" customWidth="1"/>
+    <col min="26" max="26" width="19" customWidth="1"/>
+    <col min="27" max="27" width="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13" customHeight="1">
@@ -373,110 +391,1281 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>轨迹文件</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>环境可复现等级</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Harness</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Harness 版本</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>操作系统</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>任务类型</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>任务难度</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>语言/框架</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>交付完整性</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>交付完整性 - 描述</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>指令遵循</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>指令遵循 - 描述</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>任务规划</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>任务规划 - 描述</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>推理能力</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>推理能力 - 描述</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>执行能力</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>执行能力 - 描述</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>其他问题</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>提交人</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>提交时间</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>父记录</t>
         </is>
       </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>审核备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="25.5" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>现有用户服务已经能单独启动了，请把 Kong 3.5 的路由配置补完整。通过网关访问用户注册、登录、查询和健康检查接口，直接绕过网关的地址在文档里标成开发用途；配置文件不要使用 alpine 镜像标签。</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>a0e3650c-eae4-4441-83d2-d93481346227</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>140b19ac-8361-4fea-ba31-6067b73d31df</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="str">
+        <f>=HYPERLINK("https://github.com/ljzljz520-eng/label-419/commit/7fc497b3125a29841ea8f79176db58da899d2749", "https://github.com/ljzljz520-eng/label-419/commit/7fc497b3125a29841ea8f79176db58da899d2749")</f>
+        <v>https://github.com/ljzljz520-eng/label-419/commit/7fc497b3125a29841ea8f79176db58da899d2749</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>a0e3650c-eae4-4441-83d2-d93481346227.jsonl</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>已容器化，可一键起环境</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Claude Code 2.1.263</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>MacOS/Linux</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>feature迭代</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>中等</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Kong 3.5、Docker Compose、FastAPI、Vue 3</t>
+        </is>
+      </c>
+      <c r="M2">
+        <v>4</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>三处镜像配置完成显式要求，独立复跑也成功。扣分点是未保留注册、登录、查询的网关级回归验证，也未用真实数据库服务跑完整业务链。</t>
+        </is>
+      </c>
+      <c r="O2">
+        <v>5</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>逐条检查了Kong 3.5路由、注册/登录/查询/健康四类网关访问、直连地址开发用途标记及“配置文件不要使用alpine镜像标签”约束，最终状态全部遵循，且修改范围与任务相关。</t>
+        </is>
+      </c>
+      <c r="Q2">
+        <v>4</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>依次定位项目、真实路由、前端/监控/文档和镜像标签，在编辑前形成路由/镜像/文档三项明确结论，之后完成复验和清理；不足是开头只有一句总目标，没有先列出可验收矩阵，导致中间验证多次临时调整。</t>
+        </is>
+      </c>
+      <c r="S2">
+        <v>4</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>正确把FastAPI的auth，health映射到不剥离前缀的Kong路由，并识别健康路由缺少OPTIONS，镜像迁移时也同步把apk改为 apt。
+主要不足是将mock 转发成功识别为实际业务端到端正常，虽在最终风险中主动披露，仍属于边界分析不足。</t>
+        </is>
+      </c>
+      <c r="U2">
+        <v>3</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>有高质量的批量检索、Kong真实解析、四路径代理矩阵和最终清理，但调用中出现DB模式遗漏、错误挂载、容器内缺curl、两次Admin JSON键误判，且至少一次 traceback被成功退出码掩盖</t>
+        </is>
+      </c>
+      <c r="W2"/>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>梁甲正</t>
+        </is>
+      </c>
+      <c r="Y2" s="3">
+        <v>46272.9375</v>
+      </c>
+      <c r="Z2"/>
+      <c r="AA2"/>
+    </row>
+    <row r="3" ht="25.5" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>从0做一个连锁门店账号中心。拆出用户服务和门店服务，网关统一转发，前端提供门店员工登录、账号管理、角色分配和门店资料页；每个服务独立数据库模式。需要容器编排、健康检查、接口文档和测试。</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>bfa84032-ba27-486c-8f72-d4a042562d01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ac84b551-a96a-40d3-8c81-c8a1abcf7a44</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="str">
+        <f>=HYPERLINK("https://github.com/ljzljz520-eng/419-0-1/commit/01a5ddc653e433b9e42ceeb53c7637547aed0c63", "https://github.com/ljzljz520-eng/419-0-1/commit/01a5ddc653e433b9e42ceeb53c7637547aed0c63")</f>
+        <v>https://github.com/ljzljz520-eng/419-0-1/commit/01a5ddc653e433b9e42ceeb53c7637547aed0c63</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>bfa84032-ba27-486c-8f72-d4a042562d01.jsonl</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>已容器化，可一键起环境</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Claude Code 2.1.263</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>MacOS/Linux</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0-1代码生成</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Node.js、Express、SQLite、Nginx、 JavaScript、HTML、CSS、Docker Compose</t>
+        </is>
+      </c>
+      <c r="M3">
+        <v>3</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>核心服务、前端、网关、Compose 和文档真实存在且可运行，两个测试套件通过；但存在员工列表越权、店长跨店迁移和停用后旧令牌仍可用的问题。</t>
+        </is>
+      </c>
+      <c r="O3">
+        <v>4</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>已逐项实现“用户服务、门店服务、网关统一转发、前端登录/账号/角色/门店资料、独立数据库、容器编排、健康检查、接口文档和测试”；但隐含的角色隔离未完全遵守</t>
+        </is>
+      </c>
+      <c r="Q3">
+        <v>4</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>先检查空目录和工具版本，再拆成6个任务并用 TaskUpdate按服务、测试、网关、前端、编排推进，阶段状态基本清晰，但是没有在权限矩阵和安全验收上处理关键歧义，遗漏了高风险负向测试。</t>
+        </is>
+      </c>
+      <c r="S3">
+        <v>3</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>能根据Node 26/better-sqlite3报错升级依赖和镜像，也能发现Nginx无尾斜杠重定向丢认证头；但没有从“门店隔离”和“停用账号”推导列表过滤、令牌撤销、跨店迁移约束，属于推理覆盖不足。</t>
+        </is>
+      </c>
+      <c r="U3">
+        <v>3</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>能从依赖、测试和镜像失败中恢复，但存在多次失败重试，且容器测试并未执行测试套件，最后的完成声明超出了该命令能证明的范围。</t>
+        </is>
+      </c>
+      <c r="W3"/>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>梁甲正</t>
+        </is>
+      </c>
+      <c r="Y3" s="3">
+        <v>46272.9625</v>
+      </c>
+      <c r="Z3"/>
+      <c r="AA3"/>
+    </row>
+    <row r="4" ht="25.5" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>当前多个进程或不同刷新入口同时运行时，同一个 Feed 可能被重复刷新，并且如果刷新过程较慢、失败或进程退出，也缺少可靠的任务恢复机制。请你为 Feed 刷新增加基于 PostgreSQL 的任务协调机制，实现使用数据库原子领取任务，并保证同一个 Feed 同时只有一个有效刷新任务，另外通过租约续期和过期接管处理长时间任务、失败和进程退出，旧租约失效后不能覆盖新任务的结果。后台调度、Worker、CLI、API、分类刷新和 UI 刷新都必须使用这套机制，同时保留现有的缓存请求、304、限流、失败重试、禁用 Feed、解析错误上限、batchSize 和 limitPerHost 行为，并补充必要的数据库迁移、配置和清理逻辑。</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>59d7e33e-a979-4c32-97eb-3d4d155f0527</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>8ccd9415-f6c1-4c19-b5a6-f20a92d6dc7d</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="str">
+        <f>=HYPERLINK("https://github.com/Xiang1218-Yu/miniflux/commit/a84533db6ca0a2ff9a47800fbf0326be6d9b3170", "https://github.com/Xiang1218-Yu/miniflux/commit/a84533db6ca0a2ff9a47800fbf0326be6d9b3170")</f>
+        <v>https://github.com/Xiang1218-Yu/miniflux/commit/a84533db6ca0a2ff9a47800fbf0326be6d9b3170</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>59d7e33e-a979-4c32-97eb-3d4d155f0527.jsonl</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>已容器化，可一键起环境</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2.1.241</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>MacOS/Linux</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>feature迭代</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Go, PostgreSQL</t>
+        </is>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>当前复核中 go test -race、go build ./...、go vet ./... 均通过，但 internal/storage/feed.go:340-431 等写入 SQL 没有 token 条件，核心隔离要求仍存在竞态。</t>
+        </is>
+      </c>
+      <c r="O4">
+        <v>3</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>已覆盖迁移、配置、清理、租约领取和续期等要求，但提示词明确要求旧租约不能覆盖新结果，实际只在内存层检查 stillOwner，未形成数据库级约束。</t>
+        </is>
+      </c>
+      <c r="Q4">
+        <v>3</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>规划阶段拆分了入口、存储、迁移、配置和测试，但没有把“所有副作用写入必须携带 token”列为验收项，也没有安排刷新流程级接管测试。</t>
+        </is>
+      </c>
+      <c r="S4">
+        <v>3</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>遇到 PostgreSQL operator does not exist: timestamp with time zone &lt; interval 后改用 make_interval 并通过测试，但将本地标志等同于数据库 fencing，同时未识别检查与写入之间的并发窗口。</t>
+        </is>
+      </c>
+      <c r="U4">
+        <v>3</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>会话中多次重复读取 handler.go，并经历一次租约 SQL 类型错误，虽然完成了纠正和基础验证，但未执行覆盖旧任务写入隔离的端到端测试。</t>
+        </is>
+      </c>
+      <c r="W4"/>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>叶琪</t>
+        </is>
+      </c>
+      <c r="Y4" s="3">
+        <v>46272.98055555556</v>
+      </c>
+      <c r="Z4"/>
+      <c r="AA4"/>
+    </row>
+    <row r="5" ht="25.5" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>在这个 WordVault 划词插件里把生词本重做一个完整的生词管理系统，替换现在的弹出页，并实现以下功能：
+1. 弹出页改成带侧边导航的面板，分总览、单词列表、复习、导入导出、设置几页，用状态切换，不重开弹窗。
+2. 总览给统计：累计收集词数、今天新增、今天复习次数、总查询次数，以及按词性分布的占比条。
+3. 单词列表支持搜索、按词性筛选、按字母或查询次数或最近更新时间排序，分页每页 20 条。每条可展开看完整信息，能改翻译、删自定义笔记、删词。
+4. 复习用间隔重复算法，别一次全出。队列做成卡片，先显示英文，回想后点开看释义和例句，再选认识、模糊、不认识，不同选择影响下次出现时间。排期用有依据的公式（类似 SM-2 简化版），不要固定间隔。
+5. 单词支持打标签、分组（如阅读来源、主题），列表和复习都能按标签过滤。
+6. 导出支持 JSON 和 CSV，导入能合并去重，重复单词不覆盖原有笔记。
+7. 单词可朗读，用 Web Speech API，英式、美式可切换。
+8. 翻译目标不写死 zh-CN，做成可配置，默认中文，设置里能换日语、韩语等。
+9. 整段划词现在只能翻译、查不了里面的词。改成自动按句拆开、逐句翻译，并把句子里像生词的词列出来，点一下收进生词本。
+10. 数据继续用现有 Dexie，升级后原记录不能丢；别破坏 Alt+Q 划词翻译逻辑。
+背景：插件是 MV3 架构，background 是 service worker，走 chrome.runtime.sendMessage 通信；弹窗和划词卡片共用同一个 Dexie 库，保持这个关系。</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>91598858-1626-4537-a317-e397e3aaf56d</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>cf4de94b-6fdd-4cb4-bcab-1d52076677ee</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="str">
+        <f>=HYPERLINK("https://github.com/qianmo317/claudccode-solocc-0001/commit/c9b2bf218d12f72d8b6cf9a8715f7b07a96ff3be", "https://github.com/qianmo317/claudccode-solocc-0001/commit/c9b2bf218d12f72d8b6cf9a8715f7b07a96ff3be")</f>
+        <v>https://github.com/qianmo317/claudccode-solocc-0001/commit/c9b2bf218d12f72d8b6cf9a8715f7b07a96ff3be</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>solocc-0001-trajectory.jsonl</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>无外部依赖</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2.1.263</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>MacOS/Linux</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>0-1代码生成</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>JavaScript, Chrome MV3, Dexie</t>
+        </is>
+      </c>
+      <c r="M5">
+        <v>4</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>10 项需求全部落地且为真实工程改动：db.js 升级 Dexie v2（words 增加 pos、*tags 多值索引、due 索引，daily 统计表，upgrade 钩子对老词回填 rep/ef/interval/due/tags 不丢数据）、manifest.json 升至 2.0 并把 lib/tts.js 注入 content_scripts 与 web_accessible_resources、content.js 实现整句拆分/逐句翻译/句中实词点击收入生词本/整句+单词朗读、popup.js 实现多页导航、统计卡、检索/筛选/排序/分页、标签过滤、SM-2 复习队列与 exportJSON/exportCSV、新增 lib/tts.js（英式 en-GB/美式 en-US + 目标语言朗读）。共 7 文件 1767 行改动 + 新增 2 文件，无 TODO/stub。未发现需求级缺失；仅个别统计字段（每日查询次数、按天复习历史曲线）链路未逐一验证，属隐含小遗漏，不影响主体功能。</t>
+        </is>
+      </c>
+      <c r="O5">
+        <v>5</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>已逐条核对全部约束：保持 Alt+Q 划词翻译快捷键与原有收词链路；弹窗与划词卡片仍共用同一个 Dexie 库（v2 升级 + upgrade 钩子保住老记录）；翻译目标做成可配置 targetLang（默认 zh-CN）而非写死，voiceAccent 英式/美式可切换；沿用 MV3 架构、background 为 service worker 并走 chrome.runtime.sendMessage 通信；未引入新包/运行时依赖。无自作主张或越界改动。</t>
+        </is>
+      </c>
+      <c r="Q5">
+        <v>4</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>按模块拆解清晰且推进稳定（DB 层→清单/统计→复习队列→导入导出→内容脚本朗读），最终以「改动总览」表格逐文件说明改动。但会话内无显式计划/状态追踪存档可证（仅靠最终总览体现），属过程产物而非外部可见计划，故非满分。</t>
+        </is>
+      </c>
+      <c r="S5">
+        <v>5</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>关键点推理到位：Dexie 用 version 链 + upgrade 钩子对老记录回填 SM-2 字段与标签，避免升级丢数据；SM-2 采用 rep/ef/interval/due 标准字段排期而非固定间隔；句子 tokenize 用正则 /[A-Za-z][A-Za-z'-]*/g 覆盖字母、连字符、撇号实词并过滤为候选词；targetLang/voiceAccent 可配置并贯穿整段与单词朗读。方案正确、边界考虑充分，思考量与难度匹配。</t>
+        </is>
+      </c>
+      <c r="U5">
+        <v>4</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>实现范围较大（会话约 125 个 assistant 动作），分多文件逐步落地，并新增 lib/tts.js、popup.css；改前先读现有结构，工具调用整体高效，未见同文件被反复读取或反复重试。因题量本身大（多模块 + 数据结构升级）故调用数偏多，非最小化，属可进一步精简，给 4。</t>
+        </is>
+      </c>
+      <c r="W5"/>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>帅先伟</t>
+        </is>
+      </c>
+      <c r="Y5" s="3">
+        <v>46272.98055555556</v>
+      </c>
+      <c r="Z5"/>
+      <c r="AA5"/>
+    </row>
+    <row r="6" ht="25.5" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>轨迹分析页点击“执行事件检测”会直接保存参数并替换事件，分析人员无法先判断结果。请改成先预览、后应用：预览返回处理曲线、噪声底、有效事件和越界数量，但不能改动轨迹、事件或审计日志。确认应用时必须使用刚预览的轨迹和参数，并沿用现有事务和权限规则。切换轨迹、线路筛选或修改参数后，旧预览立即失效。预览或应用失败时保留已保存结果并提示原因，同时防止重复提交。补充测试，证明预览不写库、应用会保存参数、事件和审计记录，后端测试和前端构建也要通过。不要改无关页面，不要提交或推送代码。</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>de0a9a95-0ff1-493f-a967-12634d8241a2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>8d449569-52bb-4bce-95aa-7203c465355a</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="str">
+        <f>=HYPERLINK("https://github.com/tiezhu996/fiber-otdr-analysis-console/commit/ec6cfb83458b4530fbe5f20097097880199eba66", "https://github.com/tiezhu996/fiber-otdr-analysis-console/commit/ec6cfb83458b4530fbe5f20097097880199eba66")</f>
+        <v>https://github.com/tiezhu996/fiber-otdr-analysis-console/commit/ec6cfb83458b4530fbe5f20097097880199eba66</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>de0a9a95-0ff1-493f-a967-12634d8241a2.jsonl</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>已容器化，可一键起环境</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2.1.251</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>MacOS/Linux</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>feature迭代</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Go, Gin, GORM, Vue 3, PostgreSQL, SQLite</t>
+        </is>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>预览不写库、应用保存参数和事件并记录审计、令牌单次使用、轨迹绑定、事务失败回滚、前端预览与应用界面均已实现，后端测试、竞态检测、前端构建和容器启动通过。扣分点是 frontend/src/stores/traces.ts 的 select() 在详情请求返回后才清空预览；慢请求下点击第 2 条轨迹时，页面仍显示第 1 条轨迹的预览和可点击的应用按钮。README.md 也保留了已失效的旧检测接口。</t>
+        </is>
+      </c>
+      <c r="O6">
+        <v>4</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>模型遵守了不提交或推送代码、不改无关页面、沿用事务和权限规则、补充测试并通过后端测试和前端构建等主要约束。未满足的明确要求是切换轨迹后旧预览立即失效；最终回复声称 select() 会立即清空预览，但代码和运行态核验均证明清空发生在详情请求返回之后。</t>
+        </is>
+      </c>
+      <c r="Q6">
+        <v>4</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>实现按后端数据结构与服务、路由与权限、后端测试、前端数据层与页面、最终验证分阶段推进，过程有持续状态说明和最终总结。开头没有给出完整任务拆解，也没有把切换轨迹、切换线路、修改参数三种失效条件逐项列为验收项，因此漏掉了轨迹切换的异步边界。</t>
+        </is>
+      </c>
+      <c r="S6">
+        <v>4</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>模型正确识别预览无副作用、一次性令牌绑定、应用事务、权限复用和失败回滚等核心设计点，并能定位 SQLite 测试污染和 TypeScript 类型问题后修正。扣分点是忽略 await 前后的异步状态边界，把请求完成后清空误判成点击后立即失效，最终总结也延续了该错误判断。</t>
+        </is>
+      </c>
+      <c r="U6">
+        <v>3</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>模型能从测试污染、类型错误和格式问题中恢复并完成验证，但工具调用明显冗余。原生轨迹共 91 次工具调用，其中 54 次 Read 只涉及 29 个唯一文件，多出 25 次重复读取；23 个文件被重复打开，frontend/src/api/client.ts 和 internal/algorithm/denoise.go 各读取 3 次。gofmt -l 已列出两个待格式化文件时，命令仍输出 gofmt clean，虽然后续修正，但过程信息不准确。</t>
+        </is>
+      </c>
+      <c r="W6"/>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>刘东</t>
+        </is>
+      </c>
+      <c r="Y6" s="3">
+        <v>46272.98055555556</v>
+      </c>
+      <c r="Z6"/>
+      <c r="AA6"/>
+    </row>
+    <row r="7" ht="25.5" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>在这个英语听力 App 上做一轮精听和跟读相关的功能迭代，尽量不破坏现有结构：
+跟读模式：播到某一行停住，留几秒跟读再自动继续下一行；设置里可调每行停留时长、跟读遍数。跟读能录音，回放对比，录音只留本地。
+精听 AB 循环：选定一句设 A、B，在 A 到 B 之间循环，循环次数可调，歌词高亮跟随这一段。
+变速播放：0.5 到 2 倍，0.25 步进；变速后歌词同步不能错位，核实浏览器变速后 currentTime 与歌词对得上。
+听写模式：隐藏歌词，逐句播放，我在输入框写原句，和原词比对给正确率，错处标出；结果可存，下次续练。
+生词和句子收藏：可对任意一句标记，句子里的词收进生词列表，支持导出；最好能从 LRC 统计词频，提示高频词。
+播放历史与学习统计：记住每课上次听到哪、累计听时长，给最近 7 天听时长柱状图或日历视图。
+播放队列：多课加进队列，顺序或随机播完自动切下一课。
+现有本地上传、收藏、分类、深色模式别动；新功能要兼容手机迷你播放器形态，不只做桌面版。
+学习记录存 localStorage 或 IndexedDB，不引后端，保持纯前端、能用 Docker 起。技术栈 React + Tailwind + Vite + PWA。</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6b272268-0b55-4229-8151-4ce7676e91bd</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7cfbb0ab-bfcf-4e12-b99b-f9bea7274b91</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="str">
+        <f>=HYPERLINK("https://github.com/qianmo317/claudccode-solocc-0002/commit/9fd2abfb1f8c9ad460e4d67749c0c0bd46d3da44", "https://github.com/qianmo317/claudccode-solocc-0002/commit/9fd2abfb1f8c9ad460e4d67749c0c0bd46d3da44")</f>
+        <v>https://github.com/qianmo317/claudccode-solocc-0002/commit/9fd2abfb1f8c9ad460e4d67749c0c0bd46d3da44</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>solocc-0002-trajectory.jsonl</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>已容器化，可一键起环境</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2.1.263</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>MacOS/Linux</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>feature迭代</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>TypeScript, React 18, Vite, Tailwind CSS, idb-keyval</t>
+        </is>
+      </c>
+      <c r="M7">
+        <v>5</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>9 项需求全部落地且验证通过（tsc 通过、生产构建通过、dev server 3000 端口冒烟通过）：跟读（ShadowPanel + useAudio 状态机）、AB 循环（ModeBar + Lyrics 行按钮，段内琥珀高亮）、变速（audio.playbackRate，只改速率，currentTime 仍在媒体时间轴，歌词不错位）、听写（DictationView，词级 LCS 比对+正确率，错处标注，结果可续练）、生词/句子收藏（停用词过滤、按词去重、导出 CSV/TXT、LRC 词频建议高频未收词）、历史统计（StatsChart，近 7 天柱状图+统计卡）、播放队列（QueuePanel，顺序/随机，onTrackEnded 驱动）、移动端（迷你条状态文字+全屏抽屉接入）。上传/收藏/分类/深色模式逻辑未动（5 改 + 10 新增文件）。无需求级缺失。</t>
+        </is>
+      </c>
+      <c r="O7">
+        <v>5</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>已逐条核对全部约束：本地上传/收藏/分类/深色模式逻辑未动；跟读录音只在本地（IndexedDB recordings.ts）；不引后端，学习记录全在 localStorage/IndexedDB；保留 Docker（compose up + 卷挂载热更）；新功能兼容手机迷你播放器形态；变速用 playbackRate 保证歌词不错位；麦克风权限受限时面板给提示而非报错。无越界改动、未引入后端依赖。</t>
+        </is>
+      </c>
+      <c r="Q7">
+        <v>4</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>按功能拆解为独立组件与 hooks（ShadowPanel/ModeBar/DictationView/StatsChart/QueuePanel/StudyCenter/useRecorder/useStudyData/recordings/study），最终交付说明结构清晰；但会话内无显式计划/状态追踪存档可证（仅靠最后说明体现），故非满分。</t>
+        </is>
+      </c>
+      <c r="S7">
+        <v>5</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>关键判断到位：变速用 audio.playbackRate（不改媒体时间轴），使变速后 currentTime 仍与 LRC 时间戳对齐、歌词不错位；听写用词级 LCS 比对并区分漏词/错词/多词；生词收集做停用词过滤+按词去重；LRC 词频用于高频未收词建议；录音 Blob 只存 IndexedDB 不上传。思考量与难度匹配。</t>
+        </is>
+      </c>
+      <c r="U7">
+        <v>4</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>范围大，用独立组件/hooks 落地（5 改 + 10 新增），并跑通 tsc、生产构建、dev server 冒烟；整体高效，未见同文件反复处理或反复重试；因功能多调用数偏多，属可进一步精简，给 4。</t>
+        </is>
+      </c>
+      <c r="W7"/>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>帅先伟</t>
+        </is>
+      </c>
+      <c r="Y7" s="3">
+        <v>46272.98055555556</v>
+      </c>
+      <c r="Z7"/>
+      <c r="AA7"/>
+    </row>
+    <row r="8" ht="25.5" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>开发“城市声音地图”平台：Vue3 构建交互式地图与录音上传界面，Node.js 提供音频存储、地点标注、标签检索和评论 API。用户可探索不同街区的环境声音，按时间、主题筛选并收藏声音故事。</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>8176ff4a-4fc5-4fb3-837e-64e4554df94e</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1af3bf92-06e2-4a96-a3ac-cd25dc508e14</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="str">
+        <f>=HYPERLINK("https://github.com/StarkXiao/xcf-2/commit/f758537a852f90604d07993353248041eaa2bc62", "https://github.com/StarkXiao/xcf-2/commit/f758537a852f90604d07993353248041eaa2bc62")</f>
+        <v>https://github.com/StarkXiao/xcf-2/commit/f758537a852f90604d07993353248041eaa2bc62</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>8176ff4a-4fc5-4fb3-837e-64e4554df94e.jsonl</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>有外部依赖，未容器化</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2.1.263</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>MacOS/Linux</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>0-1代码生成</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Vue 3, Vite, Leaflet, Node.js, Express, multer</t>
+        </is>
+      </c>
+      <c r="M8">
+        <v>5</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>完成UploadModal、FilterSidebar、App.vue 和地图选点流程。`npm run build` 成功；Vite 页面和 API/audio 代理返回 200，Range 音频返回 206，几个主要组件转换也都返回 200。</t>
+        </is>
+      </c>
+      <c r="O8">
+        <v>5</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>地图、麦克风/文件上传、地点标注、标签和关键词搜索、时间/主题/收藏筛选、评论及音频存储都能在代码中找到对应实现，和原需求相符。</t>
+        </is>
+      </c>
+      <c r="Q8">
+        <v>5</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>从上轮中断的上传弹窗继续，接着完成筛选侧栏和 App.vue 连接，再处理资源释放，最后跑构建和联调检查，步骤衔接正常。</t>
+        </is>
+      </c>
+      <c r="S8">
+        <v>5</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>查明上传接口本身成功，问题来自 shell 变量混入日志；另外发现预览 object URL 每次重算都新建，补了 revoke。之后检查了只看收藏、组件编译和代理链路。</t>
+        </is>
+      </c>
+      <c r="U8">
+        <v>4</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>构建和联调命令都成功，没有新的失败构建。 shell 测试错误和 stream 中断通过恢复、重跑解决了。</t>
+        </is>
+      </c>
+      <c r="W8"/>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>肖常峰</t>
+        </is>
+      </c>
+      <c r="Y8" s="3">
+        <v>46272.98055555556</v>
+      </c>
+      <c r="Z8"/>
+      <c r="AA8"/>
+    </row>
+    <row r="9" ht="25.5" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>把现在只能查看的“规则中心”改成可配置页面：所有检测规则由后端统一提供，支持启用和停用，并将配置保存到 SQLite。新建审查时只记录已启用规则的检测结果，历史审查不能受后续配置影响；系统至少要保留一条启用规则，关闭失败时前端需提示并恢复状态。同时动态展示启用规则数，补充相关后端测试，保证现有风险豁免功能不受影响，pytest -q 和 npm run build 均能通过。</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>6c3fd7ce-b14e-4162-9c9e-a4408de6e110</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0e37222c-77af-4e04-8777-d0e8fb68208d</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="str">
+        <f>=HYPERLINK("https://github.com/makabaka-boop/contract-lens/commit/3b0c88dae13b7492cc52f4318b3b53741f83288a", "https://github.com/makabaka-boop/contract-lens/commit/3b0c88dae13b7492cc52f4318b3b53741f83288a")</f>
+        <v>https://github.com/makabaka-boop/contract-lens/commit/3b0c88dae13b7492cc52f4318b3b53741f83288a</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>6c3fd7ce-b14e-4162-9c9e-a4408de6e110.jsonl</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>无外部依赖</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2.1.263</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>MacOS/Linux</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>feature迭代</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Python, FastAPI, SQLite, pytest, TypeScript, React, Vite</t>
+        </is>
+      </c>
+      <c r="M9">
+        <v>4</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>主要功能都完成了。规则改为由后端统一返回，启停状态会保存到 SQLite；新建审查只保存启用规则产生的结果，修改配置不会影响历史记录。前端增加了规则开关、启用数量和失败回滚提示，风险豁免也有回归测试。实际复跑结果是后端 17 条测试通过，前端构建成功。但是因为前端没有捕获网络请求直接失败的情况。</t>
+        </is>
+      </c>
+      <c r="O9">
+        <v>4</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>需求里提到的功能和测试项基本都做到了，也没有改动原有风险豁免逻辑。模型额外创建并推送了 worktree-rules-config 分支，这一步题面中没有要求。</t>
+        </is>
+      </c>
+      <c r="Q9">
+        <v>5</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>开始先看了项目结构，然后按后端规则配置、测试、前端页面和最终验证几个阶段推进。过程中有更新任务状态，最后也逐项说明了实现和测试结果，整体比较清楚。</t>
+        </is>
+      </c>
+      <c r="S9">
+        <v>3</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>整体实现思路没有问题，但排查测试失败时绕了不少路。实际原因是模型把 new_json 写成了 new_value，一开始却怀疑数据库路径、sqlite3.Row 和变量遮蔽，尝试多次后才回头检查源码找到拼写错误。最后虽然修好了，但定位过程不够直接。</t>
+        </is>
+      </c>
+      <c r="U9">
+        <v>3</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>工具调用比较拖沓。围绕同一个 row_to_change 报错，连续做了临时数据库复现、逐列读取、字节码检查等十多次排查，最后发现只是字段名写错。另外还有一次 worktree 路径限制报错和一次端口占用，处理后测试及构建都通过了。</t>
+        </is>
+      </c>
+      <c r="W9"/>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>张鑫宇</t>
+        </is>
+      </c>
+      <c r="Y9" s="3">
+        <v>46272.979166666664</v>
+      </c>
+      <c r="Z9"/>
+      <c r="AA9"/>
+    </row>
+    <row r="10" ht="25.5" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>做个请假补课的功能吧。现在学员请假都是线下记，后面补没补、课时扣没扣很容易乱。
+前台能登记请假，管理员审核；审核通过后自动生成一条待补课记录。补完课以后把上课记录和剩余课时一起处理掉。
+注意别重复请假、重复审核或者重复扣课，原来的报名、排课这些功能也别受影响。核心场景自己补几个测试跑一下。</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>39bcfcc7-7c30-4c14-9b76-0cf04a027a5a</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>81e712b3-e0f3-4a06-abe2-76e0c0c45678</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="str">
+        <f>=HYPERLINK("https://github.com/zzvv/zw-21-1/commit/ff5418aa723aa585b07f1ef83cb09e52b8ec9920", "https://github.com/zzvv/zw-21-1/commit/ff5418aa723aa585b07f1ef83cb09e52b8ec9920")</f>
+        <v>https://github.com/zzvv/zw-21-1/commit/ff5418aa723aa585b07f1ef83cb09e52b8ec9920</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>39bcfcc7-7c30-4c14-9b76-0cf04a027a5a.jsonl</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>有外部依赖，未容器化</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2.1.263</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>MacOS/Linux</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>feature迭代</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Python、FastAPI、SQLAlchemy、MySQL、Vue 3、Element Plus</t>
+        </is>
+      </c>
+      <c r="M10">
+        <v>3</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>完成了请假登记、审核、生成待补课、补课扣课，以及对应前后端页面和 16 个测试。已有 MySQL 库的增量迁移没有补齐，旧表缺少 makeup_id 时可能影响上课记录。</t>
+        </is>
+      </c>
+      <c r="O10">
+        <v>3</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>登记请假、管理员审核、补课记录、课时扣减和重复操作拦截都有实现。现有数据库表结构升级没有处理完整，原有上课记录在已初始化环境下存在风险。</t>
+        </is>
+      </c>
+      <c r="Q10">
+        <v>4</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>先查看现有模型、路由、前端和依赖，再按后端、测试、前端、构建的顺序推进。中途测试失败后定位到报名状态设置冲突，并修正了测试。</t>
+        </is>
+      </c>
+      <c r="S10">
+        <v>3</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>能发现并处理请假和补课对象互相引用导致的序列化递归，也考虑了重复审核和重复扣课。没有把已有数据库的表结构迁移纳入实现，落地边界考虑不足。</t>
+        </is>
+      </c>
+      <c r="U10">
+        <v>4</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>依赖安装被 PEP 668 和网络 SSL 问题阻断后，改用内存 SQLite 和标准库 unittest 完成验证；16 个测试通过，前端构建也通过。</t>
+        </is>
+      </c>
+      <c r="W10"/>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>周伟</t>
+        </is>
+      </c>
+      <c r="Y10" s="3">
+        <v>46272.99375</v>
+      </c>
+      <c r="Z10"/>
+      <c r="AA10"/>
+    </row>
+    <row r="11" ht="25.5" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>
+客服向外部服务商提供排障数据前需统一脱敏。请建设策略编排服务：运营可在网页创建并版本化邮箱、手机号、身份证及正则规则，发布后批量处理JSONL，重复请求不得生成重复任务。任务支持并发、取消和重启续跑，异常时不能丢失进度，并记录规则命中与状态审计。用Go、React和SQLite实现API与页面，提供Docker Compose一键启动，补齐规则、恢复及端到端测试。</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2d3a3a80-de97-4b2c-9a10-61d39c8447a2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>6793483e-992b-4f35-8f94-c540c4a644eb</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="str">
+        <f>=HYPERLINK("https://github.com/fddhuwenjie/cc-redaction-orchestrator-pilot-20260907/commit/28b4aeaa5888b9fb6067f3fbbb3bc40b883ea6d4", "https://github.com/fddhuwenjie/cc-redaction-orchestrator-pilot-20260907/commit/28b4aeaa5888b9fb6067f3fbbb3bc40b883ea6d4")</f>
+        <v>https://github.com/fddhuwenjie/cc-redaction-orchestrator-pilot-20260907/commit/28b4aeaa5888b9fb6067f3fbbb3bc40b883ea6d4</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ClaudeCodeCLI_第一轮代码生成轨迹.jsonl</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>已容器化，可一键起环境</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2.1.228</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>MacOS/Linux</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>0-1代码生成</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Go 1.25、React 18、TypeScript 5.6、SQLite（modernc.org/sqlite）、Docker Compose、Playwright</t>
+        </is>
+      </c>
+      <c r="M11">
+        <v>3</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>后端测试、静态检查、并发检测和前端构建均通过，容器也能健康启动；但空数据库返回空值后，策略页面执行列表遍历即崩溃，真实端到端流程无法进入策略管理，模型仍宣称实现完成，交付需要修复后才能正常使用。</t>
+        </is>
+      </c>
+      <c r="O11">
+        <v>4</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>明确要求的技术栈、并发取消、重启续跑、幂等审计和测试均有对应实现，也未擅自更换技术方案。主要偏差是端到端测试只完成文件编写，没有在可运行的浏览器环境确认成功，存在明确验证缺口。</t>
+        </is>
+      </c>
+      <c r="Q11">
+        <v>4</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>模型按后端、前端、容器化、测试与文档逐步推进，并使用任务状态更新记录阶段，复杂任务拆解总体清楚。后半段在浏览器依赖和端到端测试上多次切换方案，排障顺序略显反复，最终也没有把页面真实可用作为完成门槛。</t>
+        </is>
+      </c>
+      <c r="S11">
+        <v>3</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>模型正确处理了幂等请求、事务串行化、批次提交、取消与重启恢复等复杂状态，并通过压力和恢复测试验证。关键不足是没有统一空集合契约，未推导出空数据库是必然首屏场景，也未从端到端失败继续定位页面崩溃根因。</t>
+        </is>
+      </c>
+      <c r="U11">
+        <v>3</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>主要构建测试均实际执行，但轨迹围绕浏览器安装、运行入口和依赖检查进行了多轮重复尝试，还出现错误工作目录与重复验证命令。最终没有跑通真实浏览器流程，工具选择与排障效率仍有明显提升空间。</t>
+        </is>
+      </c>
+      <c r="W11"/>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>胡文杰</t>
+        </is>
+      </c>
+      <c r="Y11" s="3">
+        <v>46273</v>
+      </c>
+      <c r="Z11"/>
+      <c r="AA11"/>
     </row>
   </sheetData>
+  <dataValidations count="5">
+    <dataValidation allowBlank="false" sqref="F2:F10" type="list">
+      <formula1>"无外部依赖,有外部依赖，未容器化,已容器化，可一键起环境"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="false" sqref="G2:G10" type="list">
+      <formula1>"Claude Code,Codex CLI"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="false" sqref="I2:I10" type="list">
+      <formula1>"MacOS/Linux,Windows"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="false" sqref="J2:J10" type="list">
+      <formula1>"Bug修复,0-1代码生成,feature迭代,代码理解,代码重构,工程化,代码测试"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="false" sqref="K2:K10" type="list">
+      <formula1>"简单,中等,困难,地狱"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
</xml_diff>